<commit_message>
v1.0.0 - Stable release
</commit_message>
<xml_diff>
--- a/data-raw/GBD_2021_Data_Tools_Guide/IHME_GBD_2021_A1_HIERARCHIES_Y2024M05D15.XLSX
+++ b/data-raw/GBD_2021_Data_Tools_Guide/IHME_GBD_2021_A1_HIERARCHIES_Y2024M05D15.XLSX
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dump_\WORKSPACE\CODE\R-REPOS\lemur\data-raw\GBD_2021_Data_Tools_Guide\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\CODE\R-REPOS\lemur\data-raw\GBD_2021_Data_Tools_Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1492E3D-BCAC-4C7D-8AD6-D0A179DEB582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3A3031-6D72-4DD0-A8A9-AFFB6A3BFCC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GBD 2021 Locations Hierarchy" sheetId="4" r:id="rId1"/>
@@ -6881,7 +6881,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -6923,6 +6923,12 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6972,6 +6978,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0000FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -74677,7 +74688,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q412"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -74692,9 +74702,9 @@
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="33.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="39.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" style="5" customWidth="1"/>
     <col min="15" max="15" width="10" style="5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.85546875" style="5" bestFit="1" customWidth="1"/>
   </cols>
@@ -74749,7 +74759,7 @@
         <v>1834</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>294</v>
       </c>
@@ -74781,7 +74791,7 @@
         <v>1827</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>295</v>
       </c>
@@ -74859,7 +74869,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>298</v>
       </c>
@@ -74896,7 +74906,7 @@
       <c r="P5" s="7"/>
       <c r="Q5"/>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>948</v>
       </c>
@@ -74928,7 +74938,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>949</v>
       </c>
@@ -74960,7 +74970,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>950</v>
       </c>
@@ -74992,7 +75002,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>300</v>
       </c>
@@ -75024,7 +75034,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>393</v>
       </c>
@@ -75061,7 +75071,7 @@
       <c r="P10" s="7"/>
       <c r="Q10"/>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>394</v>
       </c>
@@ -75093,7 +75103,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>395</v>
       </c>
@@ -75125,7 +75135,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>396</v>
       </c>
@@ -75157,7 +75167,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>397</v>
       </c>
@@ -75192,7 +75202,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>398</v>
       </c>
@@ -75227,7 +75237,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>399</v>
       </c>
@@ -75346,7 +75356,7 @@
       </c>
       <c r="Q18"/>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>954</v>
       </c>
@@ -75381,7 +75391,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>934</v>
       </c>
@@ -75413,7 +75423,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>946</v>
       </c>
@@ -75445,7 +75455,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>947</v>
       </c>
@@ -75477,7 +75487,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>322</v>
       </c>
@@ -75514,7 +75524,7 @@
       <c r="P23" s="7"/>
       <c r="Q23"/>
     </row>
-    <row r="24" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>328</v>
       </c>
@@ -75551,7 +75561,7 @@
       <c r="P24" s="7"/>
       <c r="Q24"/>
     </row>
-    <row r="25" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>329</v>
       </c>
@@ -75588,7 +75598,7 @@
       <c r="P25" s="7"/>
       <c r="Q25"/>
     </row>
-    <row r="26" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>1048</v>
       </c>
@@ -75673,7 +75683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>302</v>
       </c>
@@ -75710,7 +75720,7 @@
       <c r="P28" s="9"/>
       <c r="Q28"/>
     </row>
-    <row r="29" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>958</v>
       </c>
@@ -75747,7 +75757,7 @@
       <c r="P29" s="9"/>
       <c r="Q29"/>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>319</v>
       </c>
@@ -75783,7 +75793,7 @@
       <c r="O30" s="9"/>
       <c r="P30" s="9"/>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>320</v>
       </c>
@@ -75819,7 +75829,7 @@
       <c r="O31" s="9"/>
       <c r="P31" s="9"/>
     </row>
-    <row r="32" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>959</v>
       </c>
@@ -75856,7 +75866,7 @@
       <c r="P32" s="9"/>
       <c r="Q32"/>
     </row>
-    <row r="33" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>321</v>
       </c>
@@ -75982,7 +75992,7 @@
       </c>
       <c r="Q35"/>
     </row>
-    <row r="36" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>346</v>
       </c>
@@ -76019,7 +76029,7 @@
       <c r="P36" s="9"/>
       <c r="Q36"/>
     </row>
-    <row r="37" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>347</v>
       </c>
@@ -76056,7 +76066,7 @@
       <c r="P37" s="9"/>
       <c r="Q37"/>
     </row>
-    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>348</v>
       </c>
@@ -76092,7 +76102,7 @@
       <c r="O38" s="9"/>
       <c r="P38" s="9"/>
     </row>
-    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>349</v>
       </c>
@@ -76131,7 +76141,7 @@
       <c r="O39" s="9"/>
       <c r="P39" s="9"/>
     </row>
-    <row r="40" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>350</v>
       </c>
@@ -76168,7 +76178,7 @@
       <c r="P40" s="9"/>
       <c r="Q40"/>
     </row>
-    <row r="41" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>351</v>
       </c>
@@ -76205,7 +76215,7 @@
       <c r="P41" s="9"/>
       <c r="Q41"/>
     </row>
-    <row r="42" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>352</v>
       </c>
@@ -76242,7 +76252,7 @@
       <c r="P42" s="9"/>
       <c r="Q42"/>
     </row>
-    <row r="43" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>353</v>
       </c>
@@ -76279,7 +76289,7 @@
       <c r="P43" s="9"/>
       <c r="Q43"/>
     </row>
-    <row r="44" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>354</v>
       </c>
@@ -76319,7 +76329,7 @@
       <c r="P44" s="9"/>
       <c r="Q44"/>
     </row>
-    <row r="45" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>355</v>
       </c>
@@ -76359,7 +76369,7 @@
       <c r="P45" s="9"/>
       <c r="Q45"/>
     </row>
-    <row r="46" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>356</v>
       </c>
@@ -76399,7 +76409,7 @@
       <c r="P46" s="9"/>
       <c r="Q46"/>
     </row>
-    <row r="47" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>357</v>
       </c>
@@ -76436,7 +76446,7 @@
       <c r="P47" s="9"/>
       <c r="Q47"/>
     </row>
-    <row r="48" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>358</v>
       </c>
@@ -76473,7 +76483,7 @@
       <c r="P48" s="9"/>
       <c r="Q48"/>
     </row>
-    <row r="49" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>359</v>
       </c>
@@ -76510,7 +76520,7 @@
       <c r="P49" s="9"/>
       <c r="Q49"/>
     </row>
-    <row r="50" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>360</v>
       </c>
@@ -76547,7 +76557,7 @@
       <c r="P50" s="9"/>
       <c r="Q50"/>
     </row>
-    <row r="51" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>361</v>
       </c>
@@ -76583,7 +76593,7 @@
       <c r="O51" s="9"/>
       <c r="P51" s="9"/>
     </row>
-    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>362</v>
       </c>
@@ -76622,7 +76632,7 @@
       <c r="O52" s="9"/>
       <c r="P52" s="9"/>
     </row>
-    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>363</v>
       </c>
@@ -76661,7 +76671,7 @@
       <c r="O53" s="9"/>
       <c r="P53" s="9"/>
     </row>
-    <row r="54" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>364</v>
       </c>
@@ -76701,7 +76711,7 @@
       <c r="P54" s="9"/>
       <c r="Q54"/>
     </row>
-    <row r="55" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>405</v>
       </c>
@@ -76741,7 +76751,7 @@
       <c r="P55" s="9"/>
       <c r="Q55"/>
     </row>
-    <row r="56" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>843</v>
       </c>
@@ -76778,7 +76788,7 @@
       <c r="P56" s="9"/>
       <c r="Q56"/>
     </row>
-    <row r="57" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>935</v>
       </c>
@@ -76815,7 +76825,7 @@
       <c r="P57" s="9"/>
       <c r="Q57"/>
     </row>
-    <row r="58" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>936</v>
       </c>
@@ -76855,7 +76865,7 @@
       <c r="P58" s="9"/>
       <c r="Q58"/>
     </row>
-    <row r="59" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>365</v>
       </c>
@@ -76936,7 +76946,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>332</v>
       </c>
@@ -76973,7 +76983,7 @@
       <c r="P61" s="9"/>
       <c r="Q61"/>
     </row>
-    <row r="62" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>337</v>
       </c>
@@ -77010,7 +77020,7 @@
       <c r="P62" s="9"/>
       <c r="Q62"/>
     </row>
-    <row r="63" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>338</v>
       </c>
@@ -77047,7 +77057,7 @@
       <c r="P63" s="9"/>
       <c r="Q63"/>
     </row>
-    <row r="64" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>339</v>
       </c>
@@ -77084,7 +77094,7 @@
       <c r="P64" s="9"/>
       <c r="Q64"/>
     </row>
-    <row r="65" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>340</v>
       </c>
@@ -77121,7 +77131,7 @@
       <c r="P65" s="9"/>
       <c r="Q65"/>
     </row>
-    <row r="66" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>341</v>
       </c>
@@ -77158,7 +77168,7 @@
       <c r="P66" s="9"/>
       <c r="Q66"/>
     </row>
-    <row r="67" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>342</v>
       </c>
@@ -77195,7 +77205,7 @@
       <c r="P67" s="9"/>
       <c r="Q67"/>
     </row>
-    <row r="68" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>400</v>
       </c>
@@ -77232,7 +77242,7 @@
       <c r="P68" s="9"/>
       <c r="Q68"/>
     </row>
-    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>401</v>
       </c>
@@ -77268,7 +77278,7 @@
       <c r="O69" s="9"/>
       <c r="P69" s="9"/>
     </row>
-    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>402</v>
       </c>
@@ -77304,7 +77314,7 @@
       <c r="O70" s="9"/>
       <c r="P70" s="9"/>
     </row>
-    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>403</v>
       </c>
@@ -77340,7 +77350,7 @@
       <c r="O71" s="9"/>
       <c r="P71" s="9"/>
     </row>
-    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>404</v>
       </c>
@@ -77376,7 +77386,7 @@
       <c r="O72" s="9"/>
       <c r="P72" s="9"/>
     </row>
-    <row r="73" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>408</v>
       </c>
@@ -77413,7 +77423,7 @@
       <c r="P73" s="9"/>
       <c r="Q73"/>
     </row>
-    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>962</v>
       </c>
@@ -77496,7 +77506,7 @@
       </c>
       <c r="Q75"/>
     </row>
-    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>367</v>
       </c>
@@ -77532,7 +77542,7 @@
       <c r="O76" s="9"/>
       <c r="P76" s="9"/>
     </row>
-    <row r="77" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>368</v>
       </c>
@@ -77568,7 +77578,7 @@
       <c r="O77" s="9"/>
       <c r="P77" s="9"/>
     </row>
-    <row r="78" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>369</v>
       </c>
@@ -77604,7 +77614,7 @@
       <c r="O78" s="9"/>
       <c r="P78" s="9"/>
     </row>
-    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>370</v>
       </c>
@@ -77640,7 +77650,7 @@
       <c r="O79" s="9"/>
       <c r="P79" s="9"/>
     </row>
-    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>995</v>
       </c>
@@ -77676,7 +77686,7 @@
       <c r="O80" s="9"/>
       <c r="P80" s="9"/>
     </row>
-    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>374</v>
       </c>
@@ -77712,7 +77722,7 @@
       <c r="O81" s="9"/>
       <c r="P81" s="9"/>
     </row>
-    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>375</v>
       </c>
@@ -77751,7 +77761,7 @@
       <c r="O82" s="9"/>
       <c r="P82" s="9"/>
     </row>
-    <row r="83" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>376</v>
       </c>
@@ -77790,7 +77800,7 @@
       <c r="O83" s="9"/>
       <c r="P83" s="9"/>
     </row>
-    <row r="84" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>741</v>
       </c>
@@ -77829,7 +77839,7 @@
       <c r="O84" s="9"/>
       <c r="P84" s="9"/>
     </row>
-    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>379</v>
       </c>
@@ -77908,7 +77918,7 @@
       </c>
       <c r="Q86"/>
     </row>
-    <row r="87" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>381</v>
       </c>
@@ -77944,7 +77954,7 @@
       <c r="O87" s="9"/>
       <c r="P87" s="9"/>
     </row>
-    <row r="88" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>382</v>
       </c>
@@ -77980,7 +77990,7 @@
       <c r="O88" s="9"/>
       <c r="P88" s="9"/>
     </row>
-    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>383</v>
       </c>
@@ -78016,7 +78026,7 @@
       <c r="O89" s="9"/>
       <c r="P89" s="9"/>
     </row>
-    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>384</v>
       </c>
@@ -78052,7 +78062,7 @@
       <c r="O90" s="9"/>
       <c r="P90" s="9"/>
     </row>
-    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>385</v>
       </c>
@@ -78132,7 +78142,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>387</v>
       </c>
@@ -78169,7 +78179,7 @@
       <c r="P93" s="9"/>
       <c r="Q93"/>
     </row>
-    <row r="94" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>388</v>
       </c>
@@ -78209,7 +78219,7 @@
       <c r="P94" s="9"/>
       <c r="Q94"/>
     </row>
-    <row r="95" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>389</v>
       </c>
@@ -78249,7 +78259,7 @@
       <c r="P95" s="9"/>
       <c r="Q95"/>
     </row>
-    <row r="96" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>390</v>
       </c>
@@ -78289,7 +78299,7 @@
       <c r="P96" s="9"/>
       <c r="Q96"/>
     </row>
-    <row r="97" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>391</v>
       </c>
@@ -78326,7 +78336,7 @@
       <c r="P97" s="9"/>
       <c r="Q97"/>
     </row>
-    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>409</v>
       </c>
@@ -78408,7 +78418,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>444</v>
       </c>
@@ -78445,7 +78455,7 @@
       <c r="P100" s="9"/>
       <c r="Q100"/>
     </row>
-    <row r="101" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>447</v>
       </c>
@@ -78482,7 +78492,7 @@
       <c r="P101" s="9"/>
       <c r="Q101"/>
     </row>
-    <row r="102" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>450</v>
       </c>
@@ -78519,7 +78529,7 @@
       <c r="P102" s="9"/>
       <c r="Q102"/>
     </row>
-    <row r="103" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>411</v>
       </c>
@@ -78556,7 +78566,7 @@
       <c r="P103" s="9"/>
       <c r="Q103"/>
     </row>
-    <row r="104" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>414</v>
       </c>
@@ -78593,7 +78603,7 @@
       <c r="P104" s="9"/>
       <c r="Q104"/>
     </row>
-    <row r="105" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>441</v>
       </c>
@@ -78632,7 +78642,7 @@
       <c r="P105" s="7"/>
       <c r="Q105"/>
     </row>
-    <row r="106" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>417</v>
       </c>
@@ -78669,7 +78679,7 @@
       <c r="P106" s="9"/>
       <c r="Q106"/>
     </row>
-    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>418</v>
       </c>
@@ -78705,7 +78715,7 @@
       <c r="O107" s="9"/>
       <c r="P107" s="9"/>
     </row>
-    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>419</v>
       </c>
@@ -78741,7 +78751,7 @@
       <c r="O108" s="9"/>
       <c r="P108" s="9"/>
     </row>
-    <row r="109" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>420</v>
       </c>
@@ -78777,7 +78787,7 @@
       <c r="O109" s="9"/>
       <c r="P109" s="9"/>
     </row>
-    <row r="110" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>996</v>
       </c>
@@ -78813,7 +78823,7 @@
       <c r="O110" s="9"/>
       <c r="P110" s="9"/>
     </row>
-    <row r="111" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>1005</v>
       </c>
@@ -78849,7 +78859,7 @@
       <c r="O111" s="9"/>
       <c r="P111" s="9"/>
     </row>
-    <row r="112" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>421</v>
       </c>
@@ -78885,7 +78895,7 @@
       <c r="O112" s="9"/>
       <c r="P112" s="9"/>
     </row>
-    <row r="113" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>453</v>
       </c>
@@ -78922,7 +78932,7 @@
       <c r="P113" s="9"/>
       <c r="Q113"/>
     </row>
-    <row r="114" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>456</v>
       </c>
@@ -78959,7 +78969,7 @@
       <c r="P114" s="9"/>
       <c r="Q114"/>
     </row>
-    <row r="115" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>423</v>
       </c>
@@ -78996,7 +79006,7 @@
       <c r="P115" s="9"/>
       <c r="Q115"/>
     </row>
-    <row r="116" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>426</v>
       </c>
@@ -79035,7 +79045,7 @@
       <c r="P116" s="7"/>
       <c r="Q116"/>
     </row>
-    <row r="117" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>459</v>
       </c>
@@ -79072,7 +79082,7 @@
       <c r="P117" s="9"/>
       <c r="Q117"/>
     </row>
-    <row r="118" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>462</v>
       </c>
@@ -79109,7 +79119,7 @@
       <c r="P118" s="9"/>
       <c r="Q118"/>
     </row>
-    <row r="119" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>849</v>
       </c>
@@ -79145,7 +79155,7 @@
       <c r="O119" s="9"/>
       <c r="P119" s="9"/>
     </row>
-    <row r="120" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>850</v>
       </c>
@@ -79184,7 +79194,7 @@
       <c r="O120" s="9"/>
       <c r="P120" s="9"/>
     </row>
-    <row r="121" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>1011</v>
       </c>
@@ -79221,7 +79231,7 @@
       <c r="P121" s="9"/>
       <c r="Q121"/>
     </row>
-    <row r="122" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>1012</v>
       </c>
@@ -79258,7 +79268,7 @@
       <c r="P122" s="9"/>
       <c r="Q122"/>
     </row>
-    <row r="123" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>429</v>
       </c>
@@ -79295,7 +79305,7 @@
       <c r="P123" s="9"/>
       <c r="Q123"/>
     </row>
-    <row r="124" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>432</v>
       </c>
@@ -79332,7 +79342,7 @@
       <c r="P124" s="9"/>
       <c r="Q124"/>
     </row>
-    <row r="125" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>435</v>
       </c>
@@ -79369,7 +79379,7 @@
       <c r="P125" s="9"/>
       <c r="Q125"/>
     </row>
-    <row r="126" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
         <v>465</v>
       </c>
@@ -79406,7 +79416,7 @@
       <c r="P126" s="9"/>
       <c r="Q126"/>
     </row>
-    <row r="127" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>438</v>
       </c>
@@ -79443,7 +79453,7 @@
       <c r="P127" s="9"/>
       <c r="Q127"/>
     </row>
-    <row r="128" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>468</v>
       </c>
@@ -79480,7 +79490,7 @@
       <c r="P128" s="9"/>
       <c r="Q128"/>
     </row>
-    <row r="129" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
         <v>471</v>
       </c>
@@ -79517,7 +79527,7 @@
       <c r="P129" s="9"/>
       <c r="Q129"/>
     </row>
-    <row r="130" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
         <v>474</v>
       </c>
@@ -79554,7 +79564,7 @@
       <c r="P130" s="9"/>
       <c r="Q130"/>
     </row>
-    <row r="131" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>477</v>
       </c>
@@ -79591,7 +79601,7 @@
       <c r="P131" s="9"/>
       <c r="Q131"/>
     </row>
-    <row r="132" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
         <v>1008</v>
       </c>
@@ -79628,7 +79638,7 @@
       <c r="P132" s="9"/>
       <c r="Q132"/>
     </row>
-    <row r="133" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>1009</v>
       </c>
@@ -79664,7 +79674,7 @@
       <c r="O133" s="9"/>
       <c r="P133" s="9"/>
     </row>
-    <row r="134" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>1010</v>
       </c>
@@ -79700,7 +79710,7 @@
       <c r="O134" s="9"/>
       <c r="P134" s="9"/>
     </row>
-    <row r="135" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>1013</v>
       </c>
@@ -79737,7 +79747,7 @@
       <c r="P135" s="9"/>
       <c r="Q135"/>
     </row>
-    <row r="136" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
         <v>480</v>
       </c>
@@ -79774,7 +79784,7 @@
       <c r="P136" s="9"/>
       <c r="Q136"/>
     </row>
-    <row r="137" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>483</v>
       </c>
@@ -79811,7 +79821,7 @@
       <c r="P137" s="9"/>
       <c r="Q137"/>
     </row>
-    <row r="138" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="3">
         <v>484</v>
       </c>
@@ -79848,7 +79858,7 @@
       <c r="P138" s="9"/>
       <c r="Q138"/>
     </row>
-    <row r="139" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>485</v>
       </c>
@@ -79885,7 +79895,7 @@
       <c r="P139" s="9"/>
       <c r="Q139"/>
     </row>
-    <row r="140" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>1006</v>
       </c>
@@ -79921,7 +79931,7 @@
       <c r="O140" s="9"/>
       <c r="P140" s="9"/>
     </row>
-    <row r="141" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>1007</v>
       </c>
@@ -79957,7 +79967,7 @@
       <c r="O141" s="9"/>
       <c r="P141" s="9"/>
     </row>
-    <row r="142" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="3">
         <v>486</v>
       </c>
@@ -79994,7 +80004,7 @@
       <c r="P142" s="9"/>
       <c r="Q142"/>
     </row>
-    <row r="143" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3">
         <v>487</v>
       </c>
@@ -80031,7 +80041,7 @@
       <c r="P143" s="9"/>
       <c r="Q143"/>
     </row>
-    <row r="144" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>845</v>
       </c>
@@ -80067,7 +80077,7 @@
       <c r="O144" s="9"/>
       <c r="P144" s="9"/>
     </row>
-    <row r="145" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>846</v>
       </c>
@@ -80103,7 +80113,7 @@
       <c r="O145" s="9"/>
       <c r="P145" s="9"/>
     </row>
-    <row r="146" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>847</v>
       </c>
@@ -80139,7 +80149,7 @@
       <c r="O146" s="9"/>
       <c r="P146" s="9"/>
     </row>
-    <row r="147" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>848</v>
       </c>
@@ -80175,7 +80185,7 @@
       <c r="O147" s="9"/>
       <c r="P147" s="9"/>
     </row>
-    <row r="148" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>943</v>
       </c>
@@ -80211,7 +80221,7 @@
       <c r="O148" s="9"/>
       <c r="P148" s="9"/>
     </row>
-    <row r="149" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="3">
         <v>489</v>
       </c>
@@ -80248,7 +80258,7 @@
       <c r="P149" s="9"/>
       <c r="Q149"/>
     </row>
-    <row r="150" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="3">
         <v>490</v>
       </c>
@@ -80285,7 +80295,7 @@
       <c r="P150" s="9"/>
       <c r="Q150"/>
     </row>
-    <row r="151" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>964</v>
       </c>
@@ -80321,7 +80331,7 @@
       <c r="O151" s="9"/>
       <c r="P151" s="9"/>
     </row>
-    <row r="152" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>965</v>
       </c>
@@ -80360,7 +80370,7 @@
       <c r="O152" s="9"/>
       <c r="P152" s="9"/>
     </row>
-    <row r="153" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>966</v>
       </c>
@@ -80399,7 +80409,7 @@
       <c r="O153" s="9"/>
       <c r="P153" s="9"/>
     </row>
-    <row r="154" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>967</v>
       </c>
@@ -80481,7 +80491,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="156" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="3">
         <v>492</v>
       </c>
@@ -80518,7 +80528,7 @@
       <c r="P156" s="9"/>
       <c r="Q156"/>
     </row>
-    <row r="157" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
         <v>493</v>
       </c>
@@ -80557,7 +80567,7 @@
       <c r="P157" s="7"/>
       <c r="Q157"/>
     </row>
-    <row r="158" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
         <v>494</v>
       </c>
@@ -80596,7 +80606,7 @@
       <c r="P158" s="7"/>
       <c r="Q158"/>
     </row>
-    <row r="159" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>495</v>
       </c>
@@ -80632,7 +80642,7 @@
       <c r="O159" s="9"/>
       <c r="P159" s="9"/>
     </row>
-    <row r="160" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>496</v>
       </c>
@@ -80668,7 +80678,7 @@
       <c r="O160" s="9"/>
       <c r="P160" s="9"/>
     </row>
-    <row r="161" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>497</v>
       </c>
@@ -80704,7 +80714,7 @@
       <c r="O161" s="9"/>
       <c r="P161" s="9"/>
     </row>
-    <row r="162" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="3">
         <v>498</v>
       </c>
@@ -80741,7 +80751,7 @@
       <c r="P162" s="9"/>
       <c r="Q162"/>
     </row>
-    <row r="163" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3">
         <v>504</v>
       </c>
@@ -80778,7 +80788,7 @@
       <c r="P163" s="9"/>
       <c r="Q163"/>
     </row>
-    <row r="164" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>968</v>
       </c>
@@ -80814,7 +80824,7 @@
       <c r="O164" s="9"/>
       <c r="P164" s="9"/>
     </row>
-    <row r="165" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>969</v>
       </c>
@@ -80850,7 +80860,7 @@
       <c r="O165" s="9"/>
       <c r="P165" s="9"/>
     </row>
-    <row r="166" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>970</v>
       </c>
@@ -80886,7 +80896,7 @@
       <c r="O166" s="9"/>
       <c r="P166" s="9"/>
     </row>
-    <row r="167" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>499</v>
       </c>
@@ -80923,7 +80933,7 @@
       <c r="P167" s="9"/>
       <c r="Q167"/>
     </row>
-    <row r="168" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>942</v>
       </c>
@@ -80959,7 +80969,7 @@
       <c r="O168" s="9"/>
       <c r="P168" s="9"/>
     </row>
-    <row r="169" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>938</v>
       </c>
@@ -80995,7 +81005,7 @@
       <c r="O169" s="9"/>
       <c r="P169" s="9"/>
     </row>
-    <row r="170" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>944</v>
       </c>
@@ -81031,7 +81041,7 @@
       <c r="O170" s="9"/>
       <c r="P170" s="9"/>
     </row>
-    <row r="171" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="3">
         <v>1004</v>
       </c>
@@ -81068,7 +81078,7 @@
       <c r="P171" s="9"/>
       <c r="Q171"/>
     </row>
-    <row r="172" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="3">
         <v>500</v>
       </c>
@@ -81105,7 +81115,7 @@
       <c r="P172" s="9"/>
       <c r="Q172"/>
     </row>
-    <row r="173" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="3">
         <v>501</v>
       </c>
@@ -81145,7 +81155,7 @@
       <c r="P173" s="9"/>
       <c r="Q173"/>
     </row>
-    <row r="174" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="3">
         <v>502</v>
       </c>
@@ -81182,7 +81192,7 @@
       <c r="P174" s="9"/>
       <c r="Q174"/>
     </row>
-    <row r="175" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="3">
         <v>503</v>
       </c>
@@ -81219,7 +81229,7 @@
       <c r="P175" s="9"/>
       <c r="Q175"/>
     </row>
-    <row r="176" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
         <v>507</v>
       </c>
@@ -81302,7 +81312,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="178" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="3">
         <v>509</v>
       </c>
@@ -81339,7 +81349,7 @@
       <c r="P178" s="9"/>
       <c r="Q178"/>
     </row>
-    <row r="179" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="3">
         <v>510</v>
       </c>
@@ -81376,7 +81386,7 @@
       <c r="P179" s="9"/>
       <c r="Q179"/>
     </row>
-    <row r="180" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>511</v>
       </c>
@@ -81412,7 +81422,7 @@
       <c r="O180" s="9"/>
       <c r="P180" s="9"/>
     </row>
-    <row r="181" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>512</v>
       </c>
@@ -81448,7 +81458,7 @@
       <c r="O181" s="9"/>
       <c r="P181" s="9"/>
     </row>
-    <row r="182" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>513</v>
       </c>
@@ -81484,7 +81494,7 @@
       <c r="O182" s="9"/>
       <c r="P182" s="9"/>
     </row>
-    <row r="183" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>514</v>
       </c>
@@ -81520,7 +81530,7 @@
       <c r="O183" s="9"/>
       <c r="P183" s="9"/>
     </row>
-    <row r="184" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="3">
         <v>515</v>
       </c>
@@ -81557,7 +81567,7 @@
       <c r="P184" s="9"/>
       <c r="Q184"/>
     </row>
-    <row r="185" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="3">
         <v>516</v>
       </c>
@@ -81594,7 +81604,7 @@
       <c r="P185" s="9"/>
       <c r="Q185"/>
     </row>
-    <row r="186" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="3">
         <v>520</v>
       </c>
@@ -81675,7 +81685,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="188" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="3">
         <v>521</v>
       </c>
@@ -81712,7 +81722,7 @@
       <c r="P188" s="9"/>
       <c r="Q188"/>
     </row>
-    <row r="189" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>522</v>
       </c>
@@ -81748,7 +81758,7 @@
       <c r="O189" s="9"/>
       <c r="P189" s="9"/>
     </row>
-    <row r="190" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>523</v>
       </c>
@@ -81784,7 +81794,7 @@
       <c r="O190" s="9"/>
       <c r="P190" s="9"/>
     </row>
-    <row r="191" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>524</v>
       </c>
@@ -81820,7 +81830,7 @@
       <c r="O191" s="9"/>
       <c r="P191" s="9"/>
     </row>
-    <row r="192" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>971</v>
       </c>
@@ -81856,7 +81866,7 @@
       <c r="O192" s="9"/>
       <c r="P192" s="9"/>
     </row>
-    <row r="193" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>525</v>
       </c>
@@ -81892,7 +81902,7 @@
       <c r="O193" s="9"/>
       <c r="P193" s="9"/>
     </row>
-    <row r="194" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="3">
         <v>992</v>
       </c>
@@ -81929,7 +81939,7 @@
       <c r="P194" s="9"/>
       <c r="Q194"/>
     </row>
-    <row r="195" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>527</v>
       </c>
@@ -81965,7 +81975,7 @@
       <c r="O195" s="9"/>
       <c r="P195" s="9"/>
     </row>
-    <row r="196" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>528</v>
       </c>
@@ -82001,7 +82011,7 @@
       <c r="O196" s="9"/>
       <c r="P196" s="9"/>
     </row>
-    <row r="197" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>536</v>
       </c>
@@ -82040,7 +82050,7 @@
       <c r="O197" s="9"/>
       <c r="P197" s="9"/>
     </row>
-    <row r="198" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="3">
         <v>529</v>
       </c>
@@ -82077,7 +82087,7 @@
       <c r="P198" s="9"/>
       <c r="Q198"/>
     </row>
-    <row r="199" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="3">
         <v>530</v>
       </c>
@@ -82114,7 +82124,7 @@
       <c r="P199" s="9"/>
       <c r="Q199"/>
     </row>
-    <row r="200" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="3">
         <v>531</v>
       </c>
@@ -82151,7 +82161,7 @@
       <c r="P200" s="9"/>
       <c r="Q200"/>
     </row>
-    <row r="201" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="3">
         <v>532</v>
       </c>
@@ -82188,7 +82198,7 @@
       <c r="P201" s="9"/>
       <c r="Q201"/>
     </row>
-    <row r="202" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="3">
         <v>533</v>
       </c>
@@ -82225,7 +82235,7 @@
       <c r="P202" s="9"/>
       <c r="Q202"/>
     </row>
-    <row r="203" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
         <v>534</v>
       </c>
@@ -82262,7 +82272,7 @@
       <c r="P203" s="9"/>
       <c r="Q203"/>
     </row>
-    <row r="204" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="3">
         <v>535</v>
       </c>
@@ -82299,7 +82309,7 @@
       <c r="P204" s="9"/>
       <c r="Q204"/>
     </row>
-    <row r="205" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="3">
         <v>541</v>
       </c>
@@ -82380,7 +82390,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="207" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="3">
         <v>543</v>
       </c>
@@ -82417,7 +82427,7 @@
       <c r="P207" s="9"/>
       <c r="Q207"/>
     </row>
-    <row r="208" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="3">
         <v>544</v>
       </c>
@@ -82454,7 +82464,7 @@
       <c r="P208" s="9"/>
       <c r="Q208"/>
     </row>
-    <row r="209" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="3">
         <v>545</v>
       </c>
@@ -82491,7 +82501,7 @@
       <c r="P209" s="9"/>
       <c r="Q209"/>
     </row>
-    <row r="210" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="3">
         <v>546</v>
       </c>
@@ -82528,7 +82538,7 @@
       <c r="P210" s="9"/>
       <c r="Q210"/>
     </row>
-    <row r="211" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="3">
         <v>554</v>
       </c>
@@ -82565,7 +82575,7 @@
       <c r="P211" s="9"/>
       <c r="Q211"/>
     </row>
-    <row r="212" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="3">
         <v>972</v>
       </c>
@@ -82605,7 +82615,7 @@
       <c r="P212" s="9"/>
       <c r="Q212"/>
     </row>
-    <row r="213" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>547</v>
       </c>
@@ -82644,7 +82654,7 @@
       <c r="O213" s="9"/>
       <c r="P213" s="9"/>
     </row>
-    <row r="214" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>548</v>
       </c>
@@ -82683,7 +82693,7 @@
       <c r="O214" s="9"/>
       <c r="P214" s="9"/>
     </row>
-    <row r="215" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="3">
         <v>557</v>
       </c>
@@ -82764,7 +82774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="217" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="3">
         <v>559</v>
       </c>
@@ -82804,7 +82814,7 @@
       <c r="P217" s="9"/>
       <c r="Q217"/>
     </row>
-    <row r="218" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="3">
         <v>567</v>
       </c>
@@ -82844,7 +82854,7 @@
       <c r="P218" s="9"/>
       <c r="Q218"/>
     </row>
-    <row r="219" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>568</v>
       </c>
@@ -82883,7 +82893,7 @@
       <c r="O219" s="9"/>
       <c r="P219" s="9"/>
     </row>
-    <row r="220" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>569</v>
       </c>
@@ -82922,7 +82932,7 @@
       <c r="O220" s="9"/>
       <c r="P220" s="9"/>
     </row>
-    <row r="221" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="3">
         <v>570</v>
       </c>
@@ -82962,7 +82972,7 @@
       <c r="P221" s="9"/>
       <c r="Q221"/>
     </row>
-    <row r="222" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="3">
         <v>571</v>
       </c>
@@ -83002,7 +83012,7 @@
       <c r="P222" s="9"/>
       <c r="Q222"/>
     </row>
-    <row r="223" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="3">
         <v>572</v>
       </c>
@@ -83039,7 +83049,7 @@
       <c r="P223" s="9"/>
       <c r="Q223"/>
     </row>
-    <row r="224" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>573</v>
       </c>
@@ -83075,7 +83085,7 @@
       <c r="O224" s="9"/>
       <c r="P224" s="9"/>
     </row>
-    <row r="225" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>574</v>
       </c>
@@ -83114,7 +83124,7 @@
       <c r="O225" s="9"/>
       <c r="P225" s="9"/>
     </row>
-    <row r="226" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="3">
         <v>575</v>
       </c>
@@ -83154,7 +83164,7 @@
       <c r="P226" s="9"/>
       <c r="Q226"/>
     </row>
-    <row r="227" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="3">
         <v>578</v>
       </c>
@@ -83194,7 +83204,7 @@
       <c r="P227" s="9"/>
       <c r="Q227"/>
     </row>
-    <row r="228" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A228" s="3">
         <v>579</v>
       </c>
@@ -83234,7 +83244,7 @@
       <c r="P228" s="9"/>
       <c r="Q228"/>
     </row>
-    <row r="229" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="3">
         <v>582</v>
       </c>
@@ -83274,7 +83284,7 @@
       <c r="P229" s="9"/>
       <c r="Q229"/>
     </row>
-    <row r="230" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="3">
         <v>585</v>
       </c>
@@ -83358,7 +83368,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="232" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A232" s="3">
         <v>560</v>
       </c>
@@ -83395,7 +83405,7 @@
       <c r="P232" s="9"/>
       <c r="Q232"/>
     </row>
-    <row r="233" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A233" s="3">
         <v>561</v>
       </c>
@@ -83432,7 +83442,7 @@
       <c r="P233" s="9"/>
       <c r="Q233"/>
     </row>
-    <row r="234" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>562</v>
       </c>
@@ -83468,7 +83478,7 @@
       <c r="O234" s="9"/>
       <c r="P234" s="9"/>
     </row>
-    <row r="235" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>563</v>
       </c>
@@ -83504,7 +83514,7 @@
       <c r="O235" s="9"/>
       <c r="P235" s="9"/>
     </row>
-    <row r="236" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>564</v>
       </c>
@@ -83540,7 +83550,7 @@
       <c r="O236" s="9"/>
       <c r="P236" s="9"/>
     </row>
-    <row r="237" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>565</v>
       </c>
@@ -83579,7 +83589,7 @@
       <c r="O237" s="9"/>
       <c r="P237" s="9"/>
     </row>
-    <row r="238" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>566</v>
       </c>
@@ -83702,7 +83712,7 @@
       </c>
       <c r="Q240"/>
     </row>
-    <row r="241" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>975</v>
       </c>
@@ -83738,7 +83748,7 @@
       <c r="O241" s="9"/>
       <c r="P241" s="9"/>
     </row>
-    <row r="242" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>976</v>
       </c>
@@ -83774,7 +83784,7 @@
       <c r="O242" s="9"/>
       <c r="P242" s="9"/>
     </row>
-    <row r="243" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A243" s="3">
         <v>589</v>
       </c>
@@ -83811,7 +83821,7 @@
       <c r="P243" s="9"/>
       <c r="Q243"/>
     </row>
-    <row r="244" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>997</v>
       </c>
@@ -83847,7 +83857,7 @@
       <c r="O244" s="9"/>
       <c r="P244" s="9"/>
     </row>
-    <row r="245" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>998</v>
       </c>
@@ -83883,7 +83893,7 @@
       <c r="O245" s="9"/>
       <c r="P245" s="9"/>
     </row>
-    <row r="246" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>591</v>
       </c>
@@ -83919,7 +83929,7 @@
       <c r="O246" s="9"/>
       <c r="P246" s="9"/>
     </row>
-    <row r="247" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>592</v>
       </c>
@@ -83955,7 +83965,7 @@
       <c r="O247" s="9"/>
       <c r="P247" s="9"/>
     </row>
-    <row r="248" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>593</v>
       </c>
@@ -83991,7 +84001,7 @@
       <c r="O248" s="9"/>
       <c r="P248" s="9"/>
     </row>
-    <row r="249" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A249" s="3">
         <v>588</v>
       </c>
@@ -84072,7 +84082,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="251" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A251" s="3">
         <v>654</v>
       </c>
@@ -84112,7 +84122,7 @@
       <c r="P251" s="9"/>
       <c r="Q251"/>
     </row>
-    <row r="252" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>977</v>
       </c>
@@ -84151,7 +84161,7 @@
       <c r="O252" s="9"/>
       <c r="P252" s="9"/>
     </row>
-    <row r="253" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>978</v>
       </c>
@@ -84190,7 +84200,7 @@
       <c r="O253" s="9"/>
       <c r="P253" s="9"/>
     </row>
-    <row r="254" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>979</v>
       </c>
@@ -84229,7 +84239,7 @@
       <c r="O254" s="9"/>
       <c r="P254" s="9"/>
     </row>
-    <row r="255" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A255" s="3">
         <v>655</v>
       </c>
@@ -84269,7 +84279,7 @@
       <c r="P255" s="9"/>
       <c r="Q255"/>
     </row>
-    <row r="256" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="3">
         <v>980</v>
       </c>
@@ -84306,7 +84316,7 @@
       <c r="P256" s="9"/>
       <c r="Q256"/>
     </row>
-    <row r="257" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>656</v>
       </c>
@@ -84342,7 +84352,7 @@
       <c r="O257" s="9"/>
       <c r="P257" s="9"/>
     </row>
-    <row r="258" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>657</v>
       </c>
@@ -84378,7 +84388,7 @@
       <c r="O258" s="9"/>
       <c r="P258" s="9"/>
     </row>
-    <row r="259" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A259" s="3">
         <v>658</v>
       </c>
@@ -84418,7 +84428,7 @@
       <c r="P259" s="9"/>
       <c r="Q259"/>
     </row>
-    <row r="260" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A260" s="3">
         <v>659</v>
       </c>
@@ -84458,7 +84468,7 @@
       <c r="P260" s="9"/>
       <c r="Q260"/>
     </row>
-    <row r="261" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A261" s="3">
         <v>660</v>
       </c>
@@ -84498,7 +84508,7 @@
       <c r="P261" s="9"/>
       <c r="Q261"/>
     </row>
-    <row r="262" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A262" s="3">
         <v>661</v>
       </c>
@@ -84538,7 +84548,7 @@
       <c r="P262" s="9"/>
       <c r="Q262"/>
     </row>
-    <row r="263" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A263" s="3">
         <v>662</v>
       </c>
@@ -84578,7 +84588,7 @@
       <c r="P263" s="9"/>
       <c r="Q263"/>
     </row>
-    <row r="264" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A264" s="3">
         <v>663</v>
       </c>
@@ -84618,7 +84628,7 @@
       <c r="P264" s="9"/>
       <c r="Q264"/>
     </row>
-    <row r="265" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A265" s="3">
         <v>664</v>
       </c>
@@ -84658,7 +84668,7 @@
       <c r="P265" s="9"/>
       <c r="Q265"/>
     </row>
-    <row r="266" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A266" s="3">
         <v>665</v>
       </c>
@@ -84695,7 +84705,7 @@
       <c r="P266" s="9"/>
       <c r="Q266"/>
     </row>
-    <row r="267" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A267" s="3">
         <v>668</v>
       </c>
@@ -84778,7 +84788,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="269" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A269" s="3">
         <v>981</v>
       </c>
@@ -84818,7 +84828,7 @@
       <c r="P269" s="9"/>
       <c r="Q269"/>
     </row>
-    <row r="270" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>670</v>
       </c>
@@ -84857,7 +84867,7 @@
       <c r="O270" s="9"/>
       <c r="P270" s="9"/>
     </row>
-    <row r="271" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>671</v>
       </c>
@@ -84896,7 +84906,7 @@
       <c r="O271" s="9"/>
       <c r="P271" s="9"/>
     </row>
-    <row r="272" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>672</v>
       </c>
@@ -84935,7 +84945,7 @@
       <c r="O272" s="9"/>
       <c r="P272" s="9"/>
     </row>
-    <row r="273" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>999</v>
       </c>
@@ -84974,7 +84984,7 @@
       <c r="O273" s="9"/>
       <c r="P273" s="9"/>
     </row>
-    <row r="274" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>1000</v>
       </c>
@@ -85013,7 +85023,7 @@
       <c r="O274" s="9"/>
       <c r="P274" s="9"/>
     </row>
-    <row r="275" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>675</v>
       </c>
@@ -85052,7 +85062,7 @@
       <c r="O275" s="9"/>
       <c r="P275" s="9"/>
     </row>
-    <row r="276" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="3">
         <v>674</v>
       </c>
@@ -85092,7 +85102,7 @@
       <c r="P276" s="9"/>
       <c r="Q276"/>
     </row>
-    <row r="277" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A277" s="3">
         <v>679</v>
       </c>
@@ -85176,7 +85186,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="279" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A279" s="3">
         <v>627</v>
       </c>
@@ -85213,7 +85223,7 @@
       <c r="P279" s="9"/>
       <c r="Q279"/>
     </row>
-    <row r="280" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A280" s="3">
         <v>628</v>
       </c>
@@ -85253,7 +85263,7 @@
       <c r="P280" s="9"/>
       <c r="Q280"/>
     </row>
-    <row r="281" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>1014</v>
       </c>
@@ -85292,7 +85302,7 @@
       <c r="O281" s="9"/>
       <c r="P281" s="9"/>
     </row>
-    <row r="282" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>1015</v>
       </c>
@@ -85331,7 +85341,7 @@
       <c r="O282" s="9"/>
       <c r="P282" s="9"/>
     </row>
-    <row r="283" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>1016</v>
       </c>
@@ -85370,7 +85380,7 @@
       <c r="O283" s="9"/>
       <c r="P283" s="9"/>
     </row>
-    <row r="284" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>1017</v>
       </c>
@@ -85409,7 +85419,7 @@
       <c r="O284" s="9"/>
       <c r="P284" s="9"/>
     </row>
-    <row r="285" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A285" s="3">
         <v>630</v>
       </c>
@@ -85449,7 +85459,7 @@
       <c r="P285" s="9"/>
       <c r="Q285"/>
     </row>
-    <row r="286" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A286" s="3">
         <v>631</v>
       </c>
@@ -85489,7 +85499,7 @@
       <c r="P286" s="9"/>
       <c r="Q286"/>
     </row>
-    <row r="287" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A287" s="3">
         <v>632</v>
       </c>
@@ -85529,7 +85539,7 @@
       <c r="P287" s="9"/>
       <c r="Q287"/>
     </row>
-    <row r="288" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A288" s="3">
         <v>639</v>
       </c>
@@ -85610,7 +85620,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="290" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A290" s="3">
         <v>641</v>
       </c>
@@ -85647,7 +85657,7 @@
       <c r="P290" s="9"/>
       <c r="Q290"/>
     </row>
-    <row r="291" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>642</v>
       </c>
@@ -85683,7 +85693,7 @@
       <c r="O291" s="9"/>
       <c r="P291" s="9"/>
     </row>
-    <row r="292" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>643</v>
       </c>
@@ -85719,7 +85729,7 @@
       <c r="O292" s="9"/>
       <c r="P292" s="9"/>
     </row>
-    <row r="293" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>644</v>
       </c>
@@ -85755,7 +85765,7 @@
       <c r="O293" s="9"/>
       <c r="P293" s="9"/>
     </row>
-    <row r="294" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>645</v>
       </c>
@@ -85791,7 +85801,7 @@
       <c r="O294" s="9"/>
       <c r="P294" s="9"/>
     </row>
-    <row r="295" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>646</v>
       </c>
@@ -85830,7 +85840,7 @@
       <c r="O295" s="9"/>
       <c r="P295" s="9"/>
     </row>
-    <row r="296" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>647</v>
       </c>
@@ -85869,7 +85879,7 @@
       <c r="O296" s="9"/>
       <c r="P296" s="9"/>
     </row>
-    <row r="297" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>648</v>
       </c>
@@ -85905,7 +85915,7 @@
       <c r="O297" s="9"/>
       <c r="P297" s="9"/>
     </row>
-    <row r="298" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>649</v>
       </c>
@@ -85941,7 +85951,7 @@
       <c r="O298" s="9"/>
       <c r="P298" s="9"/>
     </row>
-    <row r="299" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>650</v>
       </c>
@@ -85977,7 +85987,7 @@
       <c r="O299" s="9"/>
       <c r="P299" s="9"/>
     </row>
-    <row r="300" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>651</v>
       </c>
@@ -86013,7 +86023,7 @@
       <c r="O300" s="9"/>
       <c r="P300" s="9"/>
     </row>
-    <row r="301" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>652</v>
       </c>
@@ -86049,7 +86059,7 @@
       <c r="O301" s="9"/>
       <c r="P301" s="9"/>
     </row>
-    <row r="302" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A302" s="3">
         <v>594</v>
       </c>
@@ -86086,7 +86096,7 @@
       <c r="P302" s="9"/>
       <c r="Q302"/>
     </row>
-    <row r="303" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>595</v>
       </c>
@@ -86122,7 +86132,7 @@
       <c r="O303" s="9"/>
       <c r="P303" s="9"/>
     </row>
-    <row r="304" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>596</v>
       </c>
@@ -86158,7 +86168,7 @@
       <c r="O304" s="9"/>
       <c r="P304" s="9"/>
     </row>
-    <row r="305" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>597</v>
       </c>
@@ -86197,7 +86207,7 @@
       <c r="O305" s="9"/>
       <c r="P305" s="9"/>
     </row>
-    <row r="306" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>598</v>
       </c>
@@ -86236,7 +86246,7 @@
       <c r="O306" s="9"/>
       <c r="P306" s="9"/>
     </row>
-    <row r="307" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>602</v>
       </c>
@@ -86272,7 +86282,7 @@
       <c r="O307" s="9"/>
       <c r="P307" s="9"/>
     </row>
-    <row r="308" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A308" s="3">
         <v>603</v>
       </c>
@@ -86309,7 +86319,7 @@
       <c r="P308" s="9"/>
       <c r="Q308"/>
     </row>
-    <row r="309" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>604</v>
       </c>
@@ -86345,7 +86355,7 @@
       <c r="O309" s="9"/>
       <c r="P309" s="9"/>
     </row>
-    <row r="310" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>605</v>
       </c>
@@ -86384,7 +86394,7 @@
       <c r="O310" s="9"/>
       <c r="P310" s="9"/>
     </row>
-    <row r="311" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A311">
         <v>606</v>
       </c>
@@ -86423,7 +86433,7 @@
       <c r="O311" s="9"/>
       <c r="P311" s="9"/>
     </row>
-    <row r="312" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A312">
         <v>607</v>
       </c>
@@ -86459,7 +86469,7 @@
       <c r="O312" s="9"/>
       <c r="P312" s="9"/>
     </row>
-    <row r="313" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A313">
         <v>608</v>
       </c>
@@ -86495,7 +86505,7 @@
       <c r="O313" s="9"/>
       <c r="P313" s="9"/>
     </row>
-    <row r="314" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A314">
         <v>609</v>
       </c>
@@ -86534,7 +86544,7 @@
       <c r="O314" s="9"/>
       <c r="P314" s="9"/>
     </row>
-    <row r="315" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A315">
         <v>612</v>
       </c>
@@ -86570,7 +86580,7 @@
       <c r="O315" s="9"/>
       <c r="P315" s="9"/>
     </row>
-    <row r="316" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="3">
         <v>613</v>
       </c>
@@ -86607,7 +86617,7 @@
       <c r="P316" s="9"/>
       <c r="Q316"/>
     </row>
-    <row r="317" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A317">
         <v>614</v>
       </c>
@@ -86643,7 +86653,7 @@
       <c r="O317" s="9"/>
       <c r="P317" s="9"/>
     </row>
-    <row r="318" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A318">
         <v>837</v>
       </c>
@@ -86682,7 +86692,7 @@
       <c r="O318" s="9"/>
       <c r="P318" s="9"/>
     </row>
-    <row r="319" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A319">
         <v>615</v>
       </c>
@@ -86718,7 +86728,7 @@
       <c r="O319" s="9"/>
       <c r="P319" s="9"/>
     </row>
-    <row r="320" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A320">
         <v>838</v>
       </c>
@@ -86757,7 +86767,7 @@
       <c r="O320" s="9"/>
       <c r="P320" s="9"/>
     </row>
-    <row r="321" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>616</v>
       </c>
@@ -86793,7 +86803,7 @@
       <c r="O321" s="9"/>
       <c r="P321" s="9"/>
     </row>
-    <row r="322" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>839</v>
       </c>
@@ -86832,7 +86842,7 @@
       <c r="O322" s="9"/>
       <c r="P322" s="9"/>
     </row>
-    <row r="323" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>618</v>
       </c>
@@ -86868,7 +86878,7 @@
       <c r="O323" s="9"/>
       <c r="P323" s="9"/>
     </row>
-    <row r="324" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="3">
         <v>619</v>
       </c>
@@ -86905,7 +86915,7 @@
       <c r="P324" s="9"/>
       <c r="Q324"/>
     </row>
-    <row r="325" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A325" s="3">
         <v>680</v>
       </c>
@@ -86945,7 +86955,7 @@
       <c r="P325" s="9"/>
       <c r="Q325"/>
     </row>
-    <row r="326" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>681</v>
       </c>
@@ -86984,7 +86994,7 @@
       <c r="O326" s="9"/>
       <c r="P326" s="9"/>
     </row>
-    <row r="327" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>682</v>
       </c>
@@ -87023,7 +87033,7 @@
       <c r="O327" s="9"/>
       <c r="P327" s="9"/>
     </row>
-    <row r="328" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>683</v>
       </c>
@@ -87062,7 +87072,7 @@
       <c r="O328" s="9"/>
       <c r="P328" s="9"/>
     </row>
-    <row r="329" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>684</v>
       </c>
@@ -87101,7 +87111,7 @@
       <c r="O329" s="9"/>
       <c r="P329" s="9"/>
     </row>
-    <row r="330" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>685</v>
       </c>
@@ -87140,7 +87150,7 @@
       <c r="O330" s="9"/>
       <c r="P330" s="9"/>
     </row>
-    <row r="331" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A331" s="3">
         <v>686</v>
       </c>
@@ -87180,7 +87190,7 @@
       <c r="P331" s="9"/>
       <c r="Q331"/>
     </row>
-    <row r="332" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A332">
         <v>687</v>
       </c>
@@ -87262,7 +87272,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="334" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A334" s="3">
         <v>689</v>
       </c>
@@ -87299,7 +87309,7 @@
       <c r="P334" s="9"/>
       <c r="Q334"/>
     </row>
-    <row r="335" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A335">
         <v>690</v>
       </c>
@@ -87335,7 +87345,7 @@
       <c r="O335" s="9"/>
       <c r="P335" s="9"/>
     </row>
-    <row r="336" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A336">
         <v>691</v>
       </c>
@@ -87371,7 +87381,7 @@
       <c r="O336" s="9"/>
       <c r="P336" s="9"/>
     </row>
-    <row r="337" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A337">
         <v>692</v>
       </c>
@@ -87407,7 +87417,7 @@
       <c r="O337" s="9"/>
       <c r="P337" s="9"/>
     </row>
-    <row r="338" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A338">
         <v>693</v>
       </c>
@@ -87443,7 +87453,7 @@
       <c r="O338" s="9"/>
       <c r="P338" s="9"/>
     </row>
-    <row r="339" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A339">
         <v>694</v>
       </c>
@@ -87479,7 +87489,7 @@
       <c r="O339" s="9"/>
       <c r="P339" s="9"/>
     </row>
-    <row r="340" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A340" s="3">
         <v>695</v>
       </c>
@@ -87562,7 +87572,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="342" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="3">
         <v>697</v>
       </c>
@@ -87599,7 +87609,7 @@
       <c r="P342" s="9"/>
       <c r="Q342"/>
     </row>
-    <row r="343" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A343" s="3">
         <v>698</v>
       </c>
@@ -87636,7 +87646,7 @@
       <c r="P343" s="9"/>
       <c r="Q343"/>
     </row>
-    <row r="344" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A344" s="3">
         <v>699</v>
       </c>
@@ -87716,7 +87726,7 @@
       </c>
       <c r="Q345"/>
     </row>
-    <row r="346" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A346">
         <v>701</v>
       </c>
@@ -87752,7 +87762,7 @@
       <c r="O346" s="9"/>
       <c r="P346" s="9"/>
     </row>
-    <row r="347" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A347">
         <v>703</v>
       </c>
@@ -87788,7 +87798,7 @@
       <c r="O347" s="9"/>
       <c r="P347" s="9"/>
     </row>
-    <row r="348" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A348" s="3">
         <v>704</v>
       </c>
@@ -87825,7 +87835,7 @@
       <c r="P348" s="9"/>
       <c r="Q348"/>
     </row>
-    <row r="349" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A349">
         <v>705</v>
       </c>
@@ -87861,7 +87871,7 @@
       <c r="O349" s="9"/>
       <c r="P349" s="9"/>
     </row>
-    <row r="350" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A350">
         <v>707</v>
       </c>
@@ -87897,7 +87907,7 @@
       <c r="O350" s="9"/>
       <c r="P350" s="9"/>
     </row>
-    <row r="351" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A351" s="3">
         <v>708</v>
       </c>
@@ -87934,7 +87944,7 @@
       <c r="P351" s="9"/>
       <c r="Q351"/>
     </row>
-    <row r="352" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A352" s="3">
         <v>709</v>
       </c>
@@ -87971,7 +87981,7 @@
       <c r="P352" s="9"/>
       <c r="Q352"/>
     </row>
-    <row r="353" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A353">
         <v>710</v>
       </c>
@@ -88007,7 +88017,7 @@
       <c r="O353" s="9"/>
       <c r="P353" s="9"/>
     </row>
-    <row r="354" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A354">
         <v>711</v>
       </c>
@@ -88043,7 +88053,7 @@
       <c r="O354" s="9"/>
       <c r="P354" s="9"/>
     </row>
-    <row r="355" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A355" s="3">
         <v>712</v>
       </c>
@@ -88080,7 +88090,7 @@
       <c r="P355" s="9"/>
       <c r="Q355"/>
     </row>
-    <row r="356" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A356">
         <v>713</v>
       </c>
@@ -88116,7 +88126,7 @@
       <c r="O356" s="9"/>
       <c r="P356" s="9"/>
     </row>
-    <row r="357" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A357">
         <v>714</v>
       </c>
@@ -88155,7 +88165,7 @@
       <c r="O357" s="9"/>
       <c r="P357" s="9"/>
     </row>
-    <row r="358" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A358">
         <v>715</v>
       </c>
@@ -88191,7 +88201,7 @@
       <c r="O358" s="9"/>
       <c r="P358" s="9"/>
     </row>
-    <row r="359" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A359" s="3">
         <v>842</v>
       </c>
@@ -88216,10 +88226,10 @@
       <c r="J359" s="9" t="s">
         <v>1842</v>
       </c>
-      <c r="K359" s="9" t="s">
-        <v>1842</v>
-      </c>
-      <c r="L359" s="9" t="s">
+      <c r="K359" s="19" t="s">
+        <v>1347</v>
+      </c>
+      <c r="L359" s="20" t="s">
         <v>1842</v>
       </c>
       <c r="M359" s="10"/>
@@ -88272,7 +88282,7 @@
       </c>
       <c r="Q360"/>
     </row>
-    <row r="361" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A361" s="3">
         <v>1056</v>
       </c>
@@ -88399,7 +88409,7 @@
       </c>
       <c r="Q363"/>
     </row>
-    <row r="364" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A364">
         <v>721</v>
       </c>
@@ -88431,7 +88441,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="365" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A365">
         <v>723</v>
       </c>
@@ -88463,7 +88473,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="366" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A366" s="3">
         <v>724</v>
       </c>
@@ -88500,7 +88510,7 @@
       <c r="P366" s="7"/>
       <c r="Q366"/>
     </row>
-    <row r="367" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A367">
         <v>725</v>
       </c>
@@ -88532,7 +88542,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="368" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A368">
         <v>726</v>
       </c>
@@ -88564,7 +88574,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="369" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A369">
         <v>941</v>
       </c>
@@ -88599,7 +88609,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="370" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A370">
         <v>727</v>
       </c>
@@ -88631,7 +88641,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="371" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A371" s="3">
         <v>945</v>
       </c>
@@ -88668,7 +88678,7 @@
       <c r="P371" s="7"/>
       <c r="Q371"/>
     </row>
-    <row r="372" spans="1:17" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A372" s="3">
         <v>854</v>
       </c>
@@ -88705,7 +88715,7 @@
       <c r="P372" s="7"/>
       <c r="Q372"/>
     </row>
-    <row r="373" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A373" s="14">
         <v>1058</v>
       </c>
@@ -88747,7 +88757,7 @@
       </c>
       <c r="P373" s="15"/>
     </row>
-    <row r="374" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A374">
         <v>1029</v>
       </c>
@@ -88779,7 +88789,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="375" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A375">
         <v>1026</v>
       </c>
@@ -88811,7 +88821,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="376" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A376">
         <v>1027</v>
       </c>
@@ -88843,7 +88853,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="377" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A377">
         <v>1028</v>
       </c>
@@ -88875,7 +88885,7 @@
         <v>1842</v>
       </c>
     </row>
-    <row r="378" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A378">
         <v>1059</v>
       </c>
@@ -88948,39 +88958,7 @@
       <c r="K412"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P378" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="2"/>
-        <filter val="3"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="10">
-      <filters>
-        <filter val="Cardiovascular Diseases"/>
-        <filter val="Chronic Respiratory diseases"/>
-        <filter val="Diabetes mellitus"/>
-        <filter val="Enteric Infections"/>
-        <filter val="Exposure to forces of nature"/>
-        <filter val="HIV/ AIDS / STD"/>
-        <filter val="Injuries (excl. Poisonings)"/>
-        <filter val="Interpersonal Violence"/>
-        <filter val="Kidney disease (excl. Diabetes)"/>
-        <filter val="Malaria"/>
-        <filter val="Maternal disorders"/>
-        <filter val="Neglected Tropical Diseases (excl. Malaria)"/>
-        <filter val="Neonatal disorders"/>
-        <filter val="Neoplasms"/>
-        <filter val="Other Communicable"/>
-        <filter val="Other Non-Communicable"/>
-        <filter val="Poisonings"/>
-        <filter val="Respiratory Infections (excl. Tuberculosis)"/>
-        <filter val="Self-harm"/>
-        <filter val="Transport Injuries"/>
-        <filter val="Tuberculosis"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:P378" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>